<commit_message>
qa + storyboard backup
</commit_message>
<xml_diff>
--- a/guides/plans/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
+++ b/guides/plans/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="627" uniqueCount="402">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="629" uniqueCount="404">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -280,13 +280,16 @@
     <t xml:space="preserve">Message and unread/read projection correct</t>
   </si>
   <si>
+    <t xml:space="preserve">MANUAL UI + FUNCTIONAL PASS</t>
+  </si>
+  <si>
     <t xml:space="preserve">Chat/realtime E2E support</t>
   </si>
   <si>
-    <t xml:space="preserve">One message, one telemetry delta</t>
-  </si>
-  <si>
-    <t xml:space="preserve">System chat messages are excluded from Statistics message count</t>
+    <t xml:space="preserve">Continue with STAT-012; retain this unique-message oracle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Farkas Anna sent one unique ordinary message in Host Circle Ops. UI showed one bubble; API showed chat total 41-&gt;42 and exactly one matching non-system message. The real Statistics worker changed today's Messages 0-&gt;1, Communication/Messages 417-&gt;418 and Communication total 426-&gt;427. Browser screenshots at 06:53 confirmed Messages 1 and Messages 418; Ratings, Moderation and the pre-message Events value stayed stable.</t>
   </si>
   <si>
     <t xml:space="preserve">P1 66</t>
@@ -382,7 +385,7 @@
     <t xml:space="preserve">Finish controlled affinity recompute</t>
   </si>
   <si>
-    <t xml:space="preserve">Graph metrics/timeline change in predicted direction</t>
+    <t xml:space="preserve">Graph metrics/timeline change in predicted direction; prior dates stay immutable</t>
   </si>
   <si>
     <t xml:space="preserve">Matching queue returns terminal</t>
@@ -397,13 +400,16 @@
     <t xml:space="preserve">Discovery/affinity projection correct</t>
   </si>
   <si>
-    <t xml:space="preserve">AdminGraphScienceService tests</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Compare same edge set across summary and explorer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Allow telemetry worker window before refresh</t>
+    <t xml:space="preserve">DEFECT FIXED; HOT-DEPLOY RUNTIME + MANUAL STATISTICS UI PASS; AFFINITY GRAPH COMPARISON PENDING</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Historical immutability regression unit source added; dev classes hot-deploy compiled; runtime snapshot contract passed; standalone unit run intentionally not started</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compare the corresponding current edge set in Affinity Graph explorer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Initial manual refresh exposed a real defect: every Jul 22-Aug 3 point was rewritten from bridgeUsers 2-&gt;0, communities 2-&gt;1 and clusterQuality 7-&gt;3. Fix preserves stored past dates and replaces only today. Hot-deploy runtime proof compared 04:51:23 to 04:58:42: today's activeEdges changed 309-&gt;313 and recurringEdges 274-&gt;278 while all 13 prior points stayed exactly unchanged. The post-fix 07:05 browser screenshot, from the 07:03 admin snapshot after another real Refresh, reselected Jul 22 and retained Active edges 16, New edges 0, Recurring 13, Weak ties 16, Network quality 67%, and Cluster quality 3%. Manual Statistics UI retest passed; direct Affinity Graph comparison remains pending and the original FAIL evidence is retained.</t>
   </si>
   <si>
     <t xml:space="preserve">MON-011</t>
@@ -1333,14 +1339,14 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.96"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="23.53"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="73.55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="63.68"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="65.9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="73.96"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="58.95"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="129.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="76.59"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="102.03"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="15.46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="77.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="134.81"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="86.6"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="15.61"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="295.9"/>
@@ -1778,24 +1784,30 @@
         <v>85</v>
       </c>
       <c r="J10" s="0" t="s">
-        <v>53</v>
+        <v>86</v>
+      </c>
+      <c r="K10" s="1" t="n">
+        <v>46238</v>
       </c>
       <c r="L10" s="0" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="M10" s="0" t="s">
-        <v>87</v>
+        <v>88</v>
+      </c>
+      <c r="N10" s="0" t="s">
+        <v>46</v>
       </c>
       <c r="O10" s="0" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="P10" s="0" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B11" s="0" t="s">
         <v>67</v>
@@ -1804,45 +1816,45 @@
         <v>4</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F11" s="0" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I11" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="J11" s="0" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="K11" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="L11" s="0" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="M11" s="0" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="O11" s="0" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="P11" s="0" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B12" s="0" t="s">
         <v>67</v>
@@ -1851,13 +1863,13 @@
         <v>4</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="F12" s="0" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G12" s="0" t="s">
         <v>20</v>
@@ -1866,24 +1878,24 @@
         <v>72</v>
       </c>
       <c r="I12" s="0" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="J12" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L12" s="0" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="M12" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="P12" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B13" s="0" t="s">
         <v>67</v>
@@ -1892,13 +1904,13 @@
         <v>4</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F13" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G13" s="0" t="s">
         <v>20</v>
@@ -1907,74 +1919,80 @@
         <v>20</v>
       </c>
       <c r="I13" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J13" s="0" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="K13" s="1" t="n">
         <v>46232</v>
       </c>
       <c r="L13" s="0" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="M13" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="O13" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="P13" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B14" s="0" t="s">
         <v>67</v>
       </c>
       <c r="C14" s="0" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D14" s="0" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E14" s="0" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F14" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H14" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I14" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="J14" s="0" t="s">
-        <v>53</v>
+        <v>126</v>
+      </c>
+      <c r="K14" s="1" t="n">
+        <v>46238</v>
       </c>
       <c r="L14" s="0" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="M14" s="0" t="s">
-        <v>126</v>
+        <v>128</v>
+      </c>
+      <c r="N14" s="0" t="s">
+        <v>77</v>
       </c>
       <c r="O14" s="0" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="P14" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B15" s="0" t="s">
         <v>67</v>
@@ -1983,39 +2001,39 @@
         <v>50</v>
       </c>
       <c r="D15" s="0" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="E15" s="0" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="F15" s="0" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="H15" s="0" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="I15" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="J15" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L15" s="0" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="M15" s="0" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="P15" s="0" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B16" s="0" t="s">
         <v>67</v>
@@ -2024,142 +2042,142 @@
         <v>50</v>
       </c>
       <c r="D16" s="0" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="E16" s="0" t="s">
         <v>20</v>
       </c>
       <c r="F16" s="0" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="G16" s="0" t="s">
         <v>20</v>
       </c>
       <c r="H16" s="0" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="I16" s="0" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="J16" s="0" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="K16" s="1" t="n">
         <v>46232</v>
       </c>
       <c r="L16" s="0" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="M16" s="0" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="O16" s="0" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="P16" s="0" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C17" s="0" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D17" s="0" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="E17" s="0" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="F17" s="0" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="H17" s="0" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="I17" s="0" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="J17" s="0" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="L17" s="0" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="M17" s="0" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="O17" s="0" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="P17" s="0" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B18" s="0" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C18" s="0" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D18" s="0" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="E18" s="0" t="s">
         <v>20</v>
       </c>
       <c r="F18" s="0" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="G18" s="0" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="H18" s="0" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="I18" s="0" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="J18" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L18" s="0" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="M18" s="0" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="O18" s="0" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="P18" s="0" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B19" s="0" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C19" s="0" t="s">
         <v>6</v>
       </c>
       <c r="D19" s="0" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="E19" s="0" t="s">
         <v>20</v>
@@ -2168,7 +2186,7 @@
         <v>20</v>
       </c>
       <c r="G19" s="0" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="H19" s="0" t="s">
         <v>20</v>
@@ -2180,10 +2198,10 @@
         <v>53</v>
       </c>
       <c r="L19" s="0" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="M19" s="0" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="P19" s="0" t="s">
         <v>48</v>
@@ -2191,16 +2209,16 @@
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B20" s="0" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C20" s="0" t="s">
         <v>6</v>
       </c>
       <c r="D20" s="0" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="E20" s="0" t="s">
         <v>20</v>
@@ -2209,48 +2227,48 @@
         <v>20</v>
       </c>
       <c r="G20" s="0" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="H20" s="0" t="s">
         <v>20</v>
       </c>
       <c r="I20" s="0" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="J20" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L20" s="0" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="M20" s="0" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="P20" s="0" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B21" s="0" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C21" s="0" t="s">
         <v>6</v>
       </c>
       <c r="D21" s="0" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="E21" s="0" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="F21" s="0" t="s">
         <v>20</v>
       </c>
       <c r="G21" s="0" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="H21" s="0" t="s">
         <v>20</v>
@@ -2262,27 +2280,27 @@
         <v>53</v>
       </c>
       <c r="L21" s="0" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="M21" s="0" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="P21" s="0" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B22" s="0" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C22" s="0" t="s">
         <v>6</v>
       </c>
       <c r="D22" s="0" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="E22" s="0" t="s">
         <v>20</v>
@@ -2291,30 +2309,30 @@
         <v>20</v>
       </c>
       <c r="G22" s="0" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="H22" s="0" t="s">
         <v>20</v>
       </c>
       <c r="I22" s="0" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="J22" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L22" s="0" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="M22" s="0" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="P22" s="0" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B23" s="0" t="s">
         <v>67</v>
@@ -2323,48 +2341,48 @@
         <v>6</v>
       </c>
       <c r="D23" s="0" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="E23" s="0" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="F23" s="0" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="G23" s="0" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="H23" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I23" s="0" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="J23" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L23" s="0" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="M23" s="0" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="P23" s="0" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B24" s="0" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C24" s="0" t="s">
         <v>6</v>
       </c>
       <c r="D24" s="0" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="E24" s="0" t="s">
         <v>20</v>
@@ -2373,22 +2391,22 @@
         <v>20</v>
       </c>
       <c r="G24" s="0" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="H24" s="0" t="s">
         <v>20</v>
       </c>
       <c r="I24" s="0" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="J24" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L24" s="0" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="M24" s="0" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="P24" s="0" t="s">
         <v>79</v>
@@ -2396,166 +2414,166 @@
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="0" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B25" s="0" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="C25" s="0" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D25" s="0" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="E25" s="0" t="s">
         <v>20</v>
       </c>
       <c r="F25" s="0" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="G25" s="0" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="H25" s="0" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="I25" s="0" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="J25" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L25" s="0" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="M25" s="0" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="P25" s="0" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B26" s="0" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="C26" s="0" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="D26" s="0" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="E26" s="0" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="F26" s="0" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="G26" s="0" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="H26" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I26" s="0" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="J26" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L26" s="0" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="M26" s="0" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="P26" s="0" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B27" s="0" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="C27" s="0" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="D27" s="0" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="E27" s="0" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="F27" s="0" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="G27" s="0" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="H27" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I27" s="0" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="J27" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L27" s="0" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="M27" s="0" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="P27" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B28" s="0" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="C28" s="0" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="D28" s="0" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="E28" s="0" t="s">
         <v>20</v>
       </c>
       <c r="F28" s="0" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="G28" s="0" t="s">
         <v>20</v>
       </c>
       <c r="H28" s="0" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="I28" s="0" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="J28" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L28" s="0" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="M28" s="0" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="O28" s="0" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="P28" s="0" t="s">
         <v>79</v>
@@ -2563,186 +2581,186 @@
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B29" s="0" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="C29" s="0" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="D29" s="0" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="E29" s="0" t="s">
         <v>20</v>
       </c>
       <c r="F29" s="0" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="G29" s="0" t="s">
         <v>20</v>
       </c>
       <c r="H29" s="0" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="I29" s="0" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="J29" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L29" s="0" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="M29" s="0" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="O29" s="0" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="P29" s="0" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B30" s="0" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="C30" s="0" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="D30" s="0" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="E30" s="0" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="F30" s="0" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="G30" s="0" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="H30" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I30" s="0" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="J30" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L30" s="0" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="M30" s="0" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="P30" s="0" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="0" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B31" s="0" t="s">
+        <v>223</v>
+      </c>
+      <c r="C31" s="0" t="s">
+        <v>265</v>
+      </c>
+      <c r="D31" s="0" t="s">
+        <v>266</v>
+      </c>
+      <c r="E31" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="F31" s="0" t="s">
+        <v>267</v>
+      </c>
+      <c r="G31" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="H31" s="0" t="s">
+        <v>244</v>
+      </c>
+      <c r="I31" s="0" t="s">
+        <v>268</v>
+      </c>
+      <c r="J31" s="0" t="s">
+        <v>269</v>
+      </c>
+      <c r="L31" s="0" t="s">
+        <v>270</v>
+      </c>
+      <c r="M31" s="0" t="s">
+        <v>271</v>
+      </c>
+      <c r="O31" s="0" t="s">
+        <v>272</v>
+      </c>
+      <c r="P31" s="0" t="s">
         <v>221</v>
-      </c>
-      <c r="C31" s="0" t="s">
-        <v>263</v>
-      </c>
-      <c r="D31" s="0" t="s">
-        <v>264</v>
-      </c>
-      <c r="E31" s="0" t="s">
-        <v>20</v>
-      </c>
-      <c r="F31" s="0" t="s">
-        <v>265</v>
-      </c>
-      <c r="G31" s="0" t="s">
-        <v>20</v>
-      </c>
-      <c r="H31" s="0" t="s">
-        <v>242</v>
-      </c>
-      <c r="I31" s="0" t="s">
-        <v>266</v>
-      </c>
-      <c r="J31" s="0" t="s">
-        <v>267</v>
-      </c>
-      <c r="L31" s="0" t="s">
-        <v>268</v>
-      </c>
-      <c r="M31" s="0" t="s">
-        <v>269</v>
-      </c>
-      <c r="O31" s="0" t="s">
-        <v>270</v>
-      </c>
-      <c r="P31" s="0" t="s">
-        <v>219</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="0" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B32" s="0" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="C32" s="0" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="D32" s="0" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="E32" s="0" t="s">
         <v>20</v>
       </c>
       <c r="F32" s="0" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="G32" s="0" t="s">
         <v>20</v>
       </c>
       <c r="H32" s="0" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="I32" s="0" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="J32" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L32" s="0" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="M32" s="0" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="P32" s="0" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="0" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B33" s="0" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="C33" s="0" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D33" s="0" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="E33" s="0" t="s">
         <v>20</v>
@@ -2754,101 +2772,101 @@
         <v>20</v>
       </c>
       <c r="H33" s="0" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="I33" s="0" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="J33" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L33" s="0" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="M33" s="0" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="P33" s="0" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="0" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B34" s="0" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="C34" s="0" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="D34" s="0" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="E34" s="0" t="s">
         <v>20</v>
       </c>
       <c r="F34" s="0" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="G34" s="0" t="s">
         <v>20</v>
       </c>
       <c r="H34" s="0" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="I34" s="0" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="J34" s="0" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="K34" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="L34" s="0" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="M34" s="0" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="N34" s="0" t="s">
         <v>77</v>
       </c>
       <c r="O34" s="0" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="P34" s="0" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="0" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B35" s="0" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="C35" s="0" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="D35" s="0" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="E35" s="0" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="F35" s="0" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="G35" s="0" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="H35" s="0" t="s">
         <v>26</v>
       </c>
       <c r="I35" s="0" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="J35" s="0" t="s">
         <v>43</v>
@@ -2857,39 +2875,39 @@
         <v>46234</v>
       </c>
       <c r="L35" s="0" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="M35" s="0" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="N35" s="0" t="s">
         <v>77</v>
       </c>
       <c r="O35" s="0" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="P35" s="0" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="0" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B36" s="0" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="C36" s="0" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="D36" s="0" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="E36" s="0" t="s">
         <v>20</v>
       </c>
       <c r="F36" s="0" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="G36" s="0" t="s">
         <v>20</v>
@@ -2898,48 +2916,48 @@
         <v>26</v>
       </c>
       <c r="I36" s="0" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="J36" s="0" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="K36" s="1" t="n">
         <v>46232</v>
       </c>
       <c r="L36" s="0" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="M36" s="0" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="N36" s="0" t="s">
         <v>77</v>
       </c>
       <c r="O36" s="0" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="P36" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="0" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B37" s="0" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="C37" s="0" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="D37" s="0" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="E37" s="0" t="s">
         <v>20</v>
       </c>
       <c r="F37" s="0" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="G37" s="0" t="s">
         <v>20</v>
@@ -2948,25 +2966,25 @@
         <v>26</v>
       </c>
       <c r="I37" s="0" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="J37" s="0" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="K37" s="1" t="n">
         <v>46232</v>
       </c>
       <c r="L37" s="0" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="M37" s="0" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="N37" s="0" t="s">
         <v>77</v>
       </c>
       <c r="O37" s="0" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="P37" s="0" t="s">
         <v>57</v>
@@ -2974,22 +2992,22 @@
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="0" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B38" s="0" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="C38" s="0" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="D38" s="0" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="E38" s="0" t="s">
         <v>20</v>
       </c>
       <c r="F38" s="0" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="G38" s="0" t="s">
         <v>20</v>
@@ -2998,48 +3016,48 @@
         <v>26</v>
       </c>
       <c r="I38" s="0" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="J38" s="0" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="K38" s="1" t="n">
         <v>46232</v>
       </c>
       <c r="L38" s="0" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="M38" s="0" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="N38" s="0" t="s">
         <v>77</v>
       </c>
       <c r="O38" s="0" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="P38" s="0" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="0" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B39" s="0" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="C39" s="0" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="D39" s="0" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="E39" s="0" t="s">
         <v>20</v>
       </c>
       <c r="F39" s="0" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="G39" s="0" t="s">
         <v>20</v>
@@ -3048,98 +3066,98 @@
         <v>26</v>
       </c>
       <c r="I39" s="0" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="J39" s="0" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="K39" s="1" t="n">
         <v>46232</v>
       </c>
       <c r="L39" s="0" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="M39" s="0" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="N39" s="0" t="s">
         <v>77</v>
       </c>
       <c r="O39" s="0" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="P39" s="0" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="0" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B40" s="0" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="C40" s="0" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="D40" s="0" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="E40" s="0" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="F40" s="0" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="G40" s="0" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="H40" s="0" t="s">
         <v>26</v>
       </c>
       <c r="I40" s="0" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="J40" s="0" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="K40" s="1" t="n">
         <v>46232</v>
       </c>
       <c r="L40" s="0" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="M40" s="0" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="N40" s="0" t="s">
         <v>77</v>
       </c>
       <c r="O40" s="0" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="P40" s="0" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="0" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="B41" s="0" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="C41" s="0" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="D41" s="0" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="E41" s="0" t="s">
         <v>20</v>
       </c>
       <c r="F41" s="0" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="G41" s="0" t="s">
         <v>20</v>
@@ -3148,222 +3166,222 @@
         <v>26</v>
       </c>
       <c r="I41" s="0" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="J41" s="0" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="K41" s="1" t="n">
         <v>46232</v>
       </c>
       <c r="L41" s="0" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="M41" s="0" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="N41" s="0" t="s">
         <v>77</v>
       </c>
       <c r="O41" s="0" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="P41" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="0" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B42" s="0" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="C42" s="0" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="D42" s="0" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="E42" s="0" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="F42" s="0" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="G42" s="0" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="H42" s="0" t="s">
         <v>26</v>
       </c>
       <c r="I42" s="0" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="J42" s="0" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="K42" s="1" t="n">
         <v>46232</v>
       </c>
       <c r="L42" s="0" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="M42" s="0" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="N42" s="0" t="s">
         <v>77</v>
       </c>
       <c r="O42" s="0" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="P42" s="0" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="0" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B43" s="0" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="C43" s="0" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="D43" s="0" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="E43" s="0" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="F43" s="0" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="G43" s="0" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="H43" s="0" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="I43" s="0" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="J43" s="0" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="K43" s="1" t="n">
         <v>46238</v>
       </c>
       <c r="L43" s="0" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="M43" s="0" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="N43" s="0" t="s">
         <v>77</v>
       </c>
       <c r="O43" s="0" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="P43" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="0" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="B44" s="0" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="C44" s="0" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="D44" s="0" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="E44" s="0" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="F44" s="0" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="G44" s="0" t="s">
         <v>20</v>
       </c>
       <c r="H44" s="0" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="I44" s="0" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="J44" s="0" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="L44" s="0" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="M44" s="0" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="O44" s="0" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="P44" s="0" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="0" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="B45" s="0" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="C45" s="0" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="D45" s="0" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="E45" s="0" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="F45" s="0" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="G45" s="0" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="H45" s="0" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="I45" s="0" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="J45" s="0" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="K45" s="1" t="n">
         <v>46238</v>
       </c>
       <c r="L45" s="0" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="M45" s="0" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="N45" s="0" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="O45" s="0" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="P45" s="0" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
admin job lag fix
</commit_message>
<xml_diff>
--- a/guides/plans/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
+++ b/guides/plans/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1164" uniqueCount="760">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1164" uniqueCount="761">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -1255,22 +1255,25 @@
     <t xml:space="preserve">Compare pointer, scroll and input frame pacing across idle UI, Admin process list, Job Detail and Chat during periodic/live updates</t>
   </si>
   <si>
-    <t xml:space="preserve">Job Detail must stay responsive during refresh; no unnecessary full-state poll or render hitch</t>
+    <t xml:space="preserve">Job Detail must stay responsive during SmartList refresh; unchanged polls must not mutate rows; only the selected changed rule may reach the detail signal</t>
   </si>
   <si>
     <t xml:space="preserve">Chat must stay responsive during WebSocket and user-realtime updates</t>
   </si>
   <si>
-    <t xml:space="preserve">OPEN â€” JOB MANUAL OBSERVED + CODE PATH CORROBORATED; CHAT REPORTED / TRACE PENDING</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UiTaskScheduler prevents overlapping polls; no trustworthy browser frame-time regression oracle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Capture 20â€“30 second Performance + Network traces for idle/list/detail/chat and correlate hitches with 5s Job polling, WebSocket events and 10/30s user realtime long-poll</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Job Detail visibly stutters and reloads the complete process-center state every 5 seconds; detailOpen is passed as unused task state, so it does not gate polling, and the component lacks OnPush. Chat shows a similar reported symptom but uses OnPush and WebSocket live events; the global user realtime scheduler is a separate 30-second poll, 10 seconds in demo. Shared root cause is unconfirmed. Both checkpoints must pass before closure.</t>
+    <t xml:space="preserve">ADMIN JOB MANUAL VISUAL PASS; PERFORMANCE TRACE + CHAT RETEST PENDING</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Focused component tests pass 6/6 for SmartList loading, keyed equality, row patching, detail isolation and local patch routing; running hot-deploy build manually showed no prior Job Detail stutter; browser frame-time trace not captured</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capture 20â€“30 second Performance + Network traces for idle/list/detail/chat; prove unchanged Job polls preserve DOM rows and non-selected updates do not re-render detail; correlate Chat hitches independently</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OPEN / PARTIAL PASS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Admin Jobs now uses SmartList-owned five-second polling, cancellation, keyed equality, visible-row patching and re-sorting with OnPush. Job Detail receives only its selected changed rule through a separate signal; the complete list is not pushed into detail. The full center remains the table data source. The 2026-08-04 hot-deployed build no longer showed the reported stutter during manual use, but no Performance trace was captured. Chat remains a separate reported symptom using OnPush, WebSocket live events and a 30-second global user realtime poll, shortened to 10 seconds in demo; its root cause remains unconfirmed. Both checkpoints must pass before closure.</t>
   </si>
   <si>
     <t xml:space="preserve">P1 65</t>
@@ -2410,13 +2413,13 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="65.9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="73.96"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="58.95"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="75.9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="127.59"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="129.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="102.03"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="15.46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="134.81"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="140.93"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="15.61"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="189.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="173.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="21.3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="295.9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="16.43"/>
   </cols>
@@ -4499,54 +4502,54 @@
         <v>415</v>
       </c>
       <c r="N46" s="0" t="s">
-        <v>404</v>
+        <v>416</v>
       </c>
       <c r="O46" s="0" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="P46" s="0" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="0" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="B47" s="0" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C47" s="0" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="D47" s="0" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="E47" s="0" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="F47" s="0" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="G47" s="0" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="H47" s="0" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="I47" s="0" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="J47" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L47" s="0" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="M47" s="0" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="O47" s="0" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="P47" s="0" t="s">
         <v>223</v>
@@ -4554,43 +4557,43 @@
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="0" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="B48" s="0" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C48" s="0" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="D48" s="0" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="E48" s="0" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="F48" s="0" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="G48" s="0" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="H48" s="0" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="I48" s="0" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="J48" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L48" s="0" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="M48" s="0" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="O48" s="0" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="P48" s="0" t="s">
         <v>140</v>
@@ -4598,43 +4601,43 @@
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="0" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="B49" s="0" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C49" s="0" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="D49" s="0" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="E49" s="0" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="F49" s="0" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="G49" s="0" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="H49" s="0" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="I49" s="0" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="J49" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L49" s="0" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="M49" s="0" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="O49" s="0" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="P49" s="0" t="s">
         <v>163</v>
@@ -4642,43 +4645,43 @@
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="0" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="B50" s="0" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C50" s="0" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="D50" s="0" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="E50" s="0" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="F50" s="0" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="G50" s="0" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="H50" s="0" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="I50" s="0" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="J50" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L50" s="0" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="M50" s="0" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="O50" s="0" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="P50" s="0" t="s">
         <v>140</v>
@@ -4686,43 +4689,43 @@
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="0" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="B51" s="0" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C51" s="0" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="D51" s="0" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="E51" s="0" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="F51" s="0" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="G51" s="0" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="H51" s="0" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="I51" s="0" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="J51" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L51" s="0" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="M51" s="0" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="O51" s="0" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="P51" s="0" t="s">
         <v>118</v>
@@ -4730,43 +4733,43 @@
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="0" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="B52" s="0" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C52" s="0" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="D52" s="0" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="E52" s="0" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="F52" s="0" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="G52" s="0" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="H52" s="0" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="I52" s="0" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="J52" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L52" s="0" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="M52" s="0" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="O52" s="0" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="P52" s="0" t="s">
         <v>150</v>
@@ -4774,43 +4777,43 @@
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="0" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="B53" s="0" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C53" s="0" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="D53" s="0" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="E53" s="0" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="F53" s="0" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="G53" s="0" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="H53" s="0" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="I53" s="0" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="J53" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L53" s="0" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="M53" s="0" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="O53" s="0" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="P53" s="0" t="s">
         <v>350</v>
@@ -4818,43 +4821,43 @@
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="0" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="B54" s="0" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C54" s="0" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="D54" s="0" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="E54" s="0" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="F54" s="0" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="G54" s="0" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="H54" s="0" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="I54" s="0" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="J54" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L54" s="0" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="M54" s="0" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="O54" s="0" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="P54" s="0" t="s">
         <v>163</v>
@@ -4862,43 +4865,43 @@
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="0" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="B55" s="0" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C55" s="0" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="D55" s="0" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="E55" s="0" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="F55" s="0" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="G55" s="0" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="H55" s="0" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="I55" s="0" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="J55" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L55" s="0" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="M55" s="0" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="O55" s="0" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="P55" s="0" t="s">
         <v>350</v>
@@ -4906,16 +4909,16 @@
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="0" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="B56" s="0" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C56" s="0" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="D56" s="0" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E56" s="0" t="s">
         <v>20</v>
@@ -4930,19 +4933,19 @@
         <v>20</v>
       </c>
       <c r="I56" s="0" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="J56" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L56" s="0" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="M56" s="0" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="O56" s="0" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="P56" s="0" t="s">
         <v>101</v>
@@ -4950,43 +4953,43 @@
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="0" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="B57" s="0" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C57" s="0" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="D57" s="0" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="E57" s="0" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="F57" s="0" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="G57" s="0" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="H57" s="0" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="I57" s="0" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="J57" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L57" s="0" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="M57" s="0" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="O57" s="0" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="P57" s="0" t="s">
         <v>163</v>
@@ -4994,16 +4997,16 @@
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="0" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="B58" s="0" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C58" s="0" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="D58" s="0" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="E58" s="0" t="s">
         <v>20</v>
@@ -5018,19 +5021,19 @@
         <v>20</v>
       </c>
       <c r="I58" s="0" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="J58" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L58" s="0" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="M58" s="0" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="O58" s="0" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="P58" s="0" t="s">
         <v>406</v>
@@ -5038,43 +5041,43 @@
     </row>
     <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="0" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="B59" s="0" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C59" s="0" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="D59" s="0" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="E59" s="0" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="F59" s="0" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="G59" s="0" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="H59" s="0" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="I59" s="0" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="J59" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L59" s="0" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="M59" s="0" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="O59" s="0" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="P59" s="0" t="s">
         <v>365</v>
@@ -5082,43 +5085,43 @@
     </row>
     <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="0" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="B60" s="0" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C60" s="0" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="D60" s="0" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="E60" s="0" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="F60" s="0" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="G60" s="0" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="H60" s="0" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="I60" s="0" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="J60" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L60" s="0" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="M60" s="0" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="O60" s="0" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="P60" s="0" t="s">
         <v>406</v>
@@ -5126,43 +5129,43 @@
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="0" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="B61" s="0" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C61" s="0" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="D61" s="0" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="E61" s="0" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="F61" s="0" t="s">
+        <v>557</v>
+      </c>
+      <c r="G61" s="0" t="s">
         <v>556</v>
       </c>
-      <c r="G61" s="0" t="s">
-        <v>555</v>
-      </c>
       <c r="H61" s="0" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="I61" s="0" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="J61" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L61" s="0" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="M61" s="0" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="O61" s="0" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="P61" s="0" t="s">
         <v>365</v>
@@ -5170,43 +5173,43 @@
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="0" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="B62" s="0" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C62" s="0" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="D62" s="0" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="E62" s="0" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="F62" s="0" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="G62" s="0" t="s">
         <v>20</v>
       </c>
       <c r="H62" s="0" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="I62" s="0" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="J62" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L62" s="0" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="M62" s="0" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="O62" s="0" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="P62" s="0" t="s">
         <v>406</v>
@@ -5214,16 +5217,16 @@
     </row>
     <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="0" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="B63" s="0" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C63" s="0" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="D63" s="0" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="E63" s="0" t="s">
         <v>20</v>
@@ -5238,19 +5241,19 @@
         <v>20</v>
       </c>
       <c r="I63" s="0" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="J63" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L63" s="0" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="M63" s="0" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="O63" s="0" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="P63" s="0" t="s">
         <v>140</v>
@@ -5258,43 +5261,43 @@
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="0" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="B64" s="0" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C64" s="0" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="D64" s="0" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="E64" s="0" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="F64" s="0" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="G64" s="0" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="H64" s="0" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="I64" s="0" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="J64" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L64" s="0" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="M64" s="0" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="O64" s="0" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="P64" s="0" t="s">
         <v>350</v>
@@ -5302,43 +5305,43 @@
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="0" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="B65" s="0" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C65" s="0" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="D65" s="0" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="E65" s="0" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="F65" s="0" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="G65" s="0" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="H65" s="0" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="I65" s="0" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="J65" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L65" s="0" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="M65" s="0" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="O65" s="0" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="P65" s="0" t="s">
         <v>140</v>
@@ -5346,22 +5349,22 @@
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="0" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="B66" s="0" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C66" s="0" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="D66" s="0" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="E66" s="0" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="F66" s="0" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="G66" s="0" t="s">
         <v>20</v>
@@ -5370,19 +5373,19 @@
         <v>20</v>
       </c>
       <c r="I66" s="0" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="J66" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L66" s="0" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="M66" s="0" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="O66" s="0" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="P66" s="0" t="s">
         <v>150</v>
@@ -5390,22 +5393,22 @@
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="0" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="B67" s="0" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C67" s="0" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="D67" s="0" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="E67" s="0" t="s">
         <v>20</v>
       </c>
       <c r="F67" s="0" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="G67" s="0" t="s">
         <v>20</v>
@@ -5414,19 +5417,19 @@
         <v>20</v>
       </c>
       <c r="I67" s="0" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="J67" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L67" s="0" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="M67" s="0" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="O67" s="0" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="P67" s="0" t="s">
         <v>185</v>
@@ -5434,43 +5437,43 @@
     </row>
     <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="0" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="B68" s="0" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C68" s="0" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="D68" s="0" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="E68" s="0" t="s">
         <v>20</v>
       </c>
       <c r="F68" s="0" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="G68" s="0" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="H68" s="0" t="s">
         <v>20</v>
       </c>
       <c r="I68" s="0" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="J68" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L68" s="0" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="M68" s="0" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="O68" s="0" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="P68" s="0" t="s">
         <v>163</v>
@@ -5478,43 +5481,43 @@
     </row>
     <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="0" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="B69" s="0" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C69" s="0" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="D69" s="0" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="E69" s="0" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="F69" s="0" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="G69" s="0" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="H69" s="0" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="I69" s="0" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="J69" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L69" s="0" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="M69" s="0" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="O69" s="0" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="P69" s="0" t="s">
         <v>150</v>
@@ -5522,16 +5525,16 @@
     </row>
     <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="0" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="B70" s="0" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C70" s="0" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="D70" s="0" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="E70" s="0" t="s">
         <v>20</v>
@@ -5546,19 +5549,19 @@
         <v>20</v>
       </c>
       <c r="I70" s="0" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="J70" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L70" s="0" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="M70" s="0" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="O70" s="0" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="P70" s="0" t="s">
         <v>350</v>
@@ -5566,19 +5569,19 @@
     </row>
     <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="0" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="B71" s="0" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C71" s="0" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="D71" s="0" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="E71" s="0" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="F71" s="0" t="s">
         <v>20</v>
@@ -5590,19 +5593,19 @@
         <v>20</v>
       </c>
       <c r="I71" s="0" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="J71" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L71" s="0" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="M71" s="0" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="O71" s="0" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="P71" s="0" t="s">
         <v>365</v>
@@ -5610,43 +5613,43 @@
     </row>
     <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="0" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="B72" s="0" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C72" s="0" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="D72" s="0" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="E72" s="0" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="F72" s="0" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="G72" s="0" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="H72" s="0" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="I72" s="0" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="J72" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L72" s="0" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="M72" s="0" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="O72" s="0" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="P72" s="0" t="s">
         <v>365</v>
@@ -5654,43 +5657,43 @@
     </row>
     <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="0" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="B73" s="0" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C73" s="0" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="D73" s="0" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="E73" s="0" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="F73" s="0" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="G73" s="0" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="H73" s="0" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="I73" s="0" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="J73" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L73" s="0" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="M73" s="0" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="O73" s="0" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="P73" s="0" t="s">
         <v>140</v>
@@ -5698,43 +5701,43 @@
     </row>
     <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="0" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="B74" s="0" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C74" s="0" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="D74" s="0" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="E74" s="0" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="F74" s="0" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="G74" s="0" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="H74" s="0" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="I74" s="0" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="J74" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L74" s="0" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="M74" s="0" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="O74" s="0" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="P74" s="0" t="s">
         <v>350</v>
@@ -5742,43 +5745,43 @@
     </row>
     <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="0" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="B75" s="0" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C75" s="0" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="D75" s="0" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="E75" s="0" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="F75" s="0" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="G75" s="0" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="H75" s="0" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="I75" s="0" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="J75" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L75" s="0" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="M75" s="0" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="O75" s="0" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="P75" s="0" t="s">
         <v>365</v>
@@ -5786,43 +5789,43 @@
     </row>
     <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="0" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="B76" s="0" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C76" s="0" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="D76" s="0" t="s">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="E76" s="0" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="F76" s="0" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="G76" s="0" t="s">
         <v>20</v>
       </c>
       <c r="H76" s="0" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="I76" s="0" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="J76" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L76" s="0" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="M76" s="0" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="O76" s="0" t="s">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="P76" s="0" t="s">
         <v>140</v>
@@ -5830,43 +5833,43 @@
     </row>
     <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="0" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="B77" s="0" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C77" s="0" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="D77" s="0" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="E77" s="0" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="F77" s="0" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="G77" s="0" t="s">
         <v>20</v>
       </c>
       <c r="H77" s="0" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="I77" s="0" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="J77" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L77" s="0" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="M77" s="0" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="O77" s="0" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="P77" s="0" t="s">
         <v>163</v>
@@ -5874,43 +5877,43 @@
     </row>
     <row r="78" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="0" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="B78" s="0" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C78" s="0" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="D78" s="0" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="E78" s="0" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="F78" s="0" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="G78" s="0" t="s">
         <v>20</v>
       </c>
       <c r="H78" s="0" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="I78" s="0" t="s">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="J78" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L78" s="0" t="s">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="M78" s="0" t="s">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="O78" s="0" t="s">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="P78" s="0" t="s">
         <v>163</v>
@@ -5918,43 +5921,43 @@
     </row>
     <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="0" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="B79" s="0" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C79" s="0" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="D79" s="0" t="s">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="E79" s="0" t="s">
         <v>20</v>
       </c>
       <c r="F79" s="0" t="s">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="G79" s="0" t="s">
         <v>20</v>
       </c>
       <c r="H79" s="0" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="I79" s="0" t="s">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="J79" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L79" s="0" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="M79" s="0" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="O79" s="0" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="P79" s="0" t="s">
         <v>406</v>
@@ -5962,43 +5965,43 @@
     </row>
     <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="0" t="s">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="B80" s="0" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C80" s="0" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="D80" s="0" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="E80" s="0" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="F80" s="0" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="G80" s="0" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="H80" s="0" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="I80" s="0" t="s">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="J80" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L80" s="0" t="s">
-        <v>730</v>
+        <v>731</v>
       </c>
       <c r="M80" s="0" t="s">
-        <v>731</v>
+        <v>732</v>
       </c>
       <c r="O80" s="0" t="s">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="P80" s="0" t="s">
         <v>163</v>
@@ -6006,16 +6009,16 @@
     </row>
     <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="0" t="s">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="B81" s="0" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C81" s="0" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="D81" s="0" t="s">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="E81" s="0" t="s">
         <v>20</v>
@@ -6030,19 +6033,19 @@
         <v>20</v>
       </c>
       <c r="I81" s="0" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="J81" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L81" s="0" t="s">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="M81" s="0" t="s">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="O81" s="0" t="s">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="P81" s="0" t="s">
         <v>350</v>
@@ -6050,43 +6053,43 @@
     </row>
     <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="0" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="B82" s="0" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C82" s="0" t="s">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="D82" s="0" t="s">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="E82" s="0" t="s">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="F82" s="0" t="s">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="G82" s="0" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="H82" s="0" t="s">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="I82" s="0" t="s">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="J82" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L82" s="0" t="s">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="M82" s="0" t="s">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="O82" s="0" t="s">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="P82" s="0" t="s">
         <v>365</v>
@@ -6094,43 +6097,43 @@
     </row>
     <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="0" t="s">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="B83" s="0" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C83" s="0" t="s">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="D83" s="0" t="s">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="E83" s="0" t="s">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="F83" s="0" t="s">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="G83" s="0" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="H83" s="0" t="s">
-        <v>755</v>
+        <v>756</v>
       </c>
       <c r="I83" s="0" t="s">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="J83" s="0" t="s">
         <v>53</v>
       </c>
       <c r="L83" s="0" t="s">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="M83" s="0" t="s">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="O83" s="0" t="s">
-        <v>759</v>
+        <v>760</v>
       </c>
       <c r="P83" s="0" t="s">
         <v>365</v>

</xml_diff>